<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-17 12:30 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -5965,7 +5965,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46189.12545385417</v>
+        <v>46190.20534189815</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>273</v>
@@ -6015,8 +6015,8 @@
       <c r="T77" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="U77" s="12" t="s">
-        <v>157</v>
+      <c r="U77" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46189.12536952546</v>
+        <v>46190.205348206015</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>278</v>
@@ -6078,8 +6078,8 @@
       <c r="T78" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="U78" s="12" t="s">
-        <v>157</v>
+      <c r="U78" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6144,7 +6144,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46189.25031092593</v>
+        <v>46190.205342534726</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>283</v>
@@ -6194,8 +6194,8 @@
       <c r="T80" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="U80" s="12" t="s">
-        <v>157</v>
+      <c r="U80" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-24 15:42 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -5143,7 +5143,7 @@
         <v>46197.59918284722</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.59920001157</v>
+        <v>46197.60713444444</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>227</v>
@@ -5450,9 +5450,11 @@
       <c r="B68" s="5">
         <v>46065.866385960646</v>
       </c>
-      <c r="C68" s="6"/>
+      <c r="C68" s="5">
+        <v>46197.607128483796</v>
+      </c>
       <c r="D68" s="5">
-        <v>46148.18533741898</v>
+        <v>46197.60726340278</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>244</v>
@@ -5497,10 +5499,10 @@
         <v>46147</v>
       </c>
       <c r="S68" s="6">
-        <v>0</v>
-      </c>
-      <c r="T68" s="12" t="s">
-        <v>82</v>
+        <v>1</v>
+      </c>
+      <c r="T68" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U68" s="11" t="s">
         <v>32</v>
@@ -5515,7 +5517,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46197.50378604166</v>
+        <v>46197.60713396991</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 13:06 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -1498,13 +1498,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46065.86638708333</v>
+        <v>46065.69972041667</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.72195689815</v>
+        <v>46092.55529023148</v>
       </c>
       <c r="D4" s="5">
-        <v>46133.77031836806</v>
+        <v>46133.603651701385</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1547,13 +1547,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46065.866387546295</v>
+        <v>46065.69972087963</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.72192355324</v>
+        <v>46092.555256886575</v>
       </c>
       <c r="D5" s="8">
-        <v>46092.72195766204</v>
+        <v>46092.55529099537</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1612,13 +1612,13 @@
         <v>33</v>
       </c>
       <c r="B6" s="5">
-        <v>46065.866388055554</v>
+        <v>46065.69972138889</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.721924108795</v>
+        <v>46092.55525744213</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.721958553244</v>
+        <v>46092.55529188657</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>34</v>
@@ -1677,13 +1677,13 @@
         <v>37</v>
       </c>
       <c r="B7" s="8">
-        <v>46065.866388587965</v>
+        <v>46065.69972192129</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.72192459491</v>
+        <v>46092.55525792824</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.72195796296</v>
+        <v>46092.555291296296</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>38</v>
@@ -1742,13 +1742,13 @@
         <v>39</v>
       </c>
       <c r="B8" s="5">
-        <v>46065.86638902778</v>
+        <v>46065.69972236111</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.721925081016</v>
+        <v>46092.55525841435</v>
       </c>
       <c r="D8" s="5">
-        <v>46100.79000630787</v>
+        <v>46100.6233396412</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>40</v>
@@ -1807,13 +1807,13 @@
         <v>42</v>
       </c>
       <c r="B9" s="8">
-        <v>46065.86638950232</v>
+        <v>46065.69972283565</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.721925879625</v>
+        <v>46092.55525921297</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.721958587965</v>
+        <v>46092.55529192129</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>43</v>
@@ -1872,11 +1872,11 @@
         <v>44</v>
       </c>
       <c r="B10" s="5">
-        <v>46065.866389999996</v>
+        <v>46065.69972333334</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46097.55431952546</v>
+        <v>46097.3876528588</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -1919,13 +1919,13 @@
         <v>47</v>
       </c>
       <c r="B11" s="8">
-        <v>46065.86639034722</v>
+        <v>46065.699723680555</v>
       </c>
       <c r="C11" s="8">
-        <v>46097.55430884259</v>
+        <v>46097.38764217593</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.55432767361</v>
+        <v>46097.38766100694</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>48</v>
@@ -1984,11 +1984,11 @@
         <v>52</v>
       </c>
       <c r="B12" s="5">
-        <v>46065.866390717594</v>
+        <v>46065.69972405092</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46137.193168541664</v>
+        <v>46137.026501875</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>53</v>
@@ -2047,13 +2047,13 @@
         <v>57</v>
       </c>
       <c r="B13" s="8">
-        <v>46065.86639111111</v>
+        <v>46065.69972444444</v>
       </c>
       <c r="C13" s="8">
-        <v>46114.522557662036</v>
+        <v>46114.35589099537</v>
       </c>
       <c r="D13" s="8">
-        <v>46114.52257165509</v>
+        <v>46114.35590498842</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>58</v>
@@ -2100,13 +2100,13 @@
         <v>60</v>
       </c>
       <c r="B14" s="5">
-        <v>46065.866385104164</v>
+        <v>46065.6997184375</v>
       </c>
       <c r="C14" s="5">
-        <v>46097.55338545139</v>
+        <v>46097.38671878472</v>
       </c>
       <c r="D14" s="5">
-        <v>46097.55340334491</v>
+        <v>46097.386736678236</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>61</v>
@@ -2165,13 +2165,13 @@
         <v>63</v>
       </c>
       <c r="B15" s="8">
-        <v>46065.86639079861</v>
+        <v>46065.69972413195</v>
       </c>
       <c r="C15" s="8">
-        <v>46107.72433622685</v>
+        <v>46107.557669560185</v>
       </c>
       <c r="D15" s="8">
-        <v>46107.72435567129</v>
+        <v>46107.55768900463</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>64</v>
@@ -2230,13 +2230,13 @@
         <v>66</v>
       </c>
       <c r="B16" s="5">
-        <v>46065.86639224537</v>
+        <v>46065.6997255787</v>
       </c>
       <c r="C16" s="5">
-        <v>46107.72438612269</v>
+        <v>46107.55771945602</v>
       </c>
       <c r="D16" s="5">
-        <v>46107.72440368056</v>
+        <v>46107.55773701389</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>67</v>
@@ -2295,13 +2295,13 @@
         <v>69</v>
       </c>
       <c r="B17" s="8">
-        <v>46065.866393055556</v>
+        <v>46065.69972638889</v>
       </c>
       <c r="C17" s="8">
-        <v>46114.522542349536</v>
+        <v>46114.35587568287</v>
       </c>
       <c r="D17" s="8">
-        <v>46114.52255778935</v>
+        <v>46114.35589112269</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>70</v>
@@ -2360,13 +2360,13 @@
         <v>73</v>
       </c>
       <c r="B18" s="5">
-        <v>46065.866393414355</v>
+        <v>46065.69972674768</v>
       </c>
       <c r="C18" s="5">
-        <v>46114.522602199075</v>
+        <v>46114.35593553241</v>
       </c>
       <c r="D18" s="5">
-        <v>46114.52262466435</v>
+        <v>46114.355957997686</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>74</v>
@@ -2413,13 +2413,13 @@
         <v>76</v>
       </c>
       <c r="B19" s="8">
-        <v>46065.866393749995</v>
+        <v>46065.69972708334</v>
       </c>
       <c r="C19" s="8">
-        <v>46097.55342099537</v>
+        <v>46097.386754328705</v>
       </c>
       <c r="D19" s="8">
-        <v>46097.55415841435</v>
+        <v>46097.387491747686</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>77</v>
@@ -2478,13 +2478,13 @@
         <v>79</v>
       </c>
       <c r="B20" s="5">
-        <v>46065.86639414352</v>
+        <v>46065.69972747685</v>
       </c>
       <c r="C20" s="5">
-        <v>46097.553338831014</v>
+        <v>46097.38667216436</v>
       </c>
       <c r="D20" s="5">
-        <v>46107.72435928241</v>
+        <v>46107.55769261574</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>80</v>
@@ -2543,13 +2543,13 @@
         <v>83</v>
       </c>
       <c r="B21" s="8">
-        <v>46065.866394571756</v>
+        <v>46065.69972790509</v>
       </c>
       <c r="C21" s="8">
-        <v>46097.55436326389</v>
+        <v>46097.38769659722</v>
       </c>
       <c r="D21" s="8">
-        <v>46097.55438569444</v>
+        <v>46097.38771902778</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>84</v>
@@ -2608,13 +2608,13 @@
         <v>86</v>
       </c>
       <c r="B22" s="5">
-        <v>46065.86639490741</v>
+        <v>46065.69972824074</v>
       </c>
       <c r="C22" s="5">
-        <v>46113.5602749074</v>
+        <v>46113.393608240745</v>
       </c>
       <c r="D22" s="5">
-        <v>46113.56027699074</v>
+        <v>46113.39361032407</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>87</v>
@@ -2673,13 +2673,13 @@
         <v>90</v>
       </c>
       <c r="B23" s="8">
-        <v>46065.86638537037</v>
+        <v>46065.699718703705</v>
       </c>
       <c r="C23" s="8">
-        <v>46114.52258550926</v>
+        <v>46114.35591884259</v>
       </c>
       <c r="D23" s="8">
-        <v>46114.52306825231</v>
+        <v>46114.35640158565</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>91</v>
@@ -2738,13 +2738,13 @@
         <v>93</v>
       </c>
       <c r="B24" s="5">
-        <v>46065.86638577546</v>
+        <v>46065.6997191088</v>
       </c>
       <c r="C24" s="5">
-        <v>46107.72465984954</v>
+        <v>46107.55799318287</v>
       </c>
       <c r="D24" s="5">
-        <v>46107.724677314814</v>
+        <v>46107.55801064815</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>94</v>
@@ -2803,11 +2803,11 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46065.86638607639</v>
+        <v>46065.69971940972</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="8">
-        <v>46174.653070949076</v>
+        <v>46174.486404282405</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2852,13 +2852,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46065.86638636574</v>
+        <v>46065.69971969907</v>
       </c>
       <c r="C26" s="5">
-        <v>46155.875902604166</v>
+        <v>46155.709235937495</v>
       </c>
       <c r="D26" s="5">
-        <v>46155.87591685185</v>
+        <v>46155.70925018519</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2917,13 +2917,13 @@
         <v>106</v>
       </c>
       <c r="B27" s="8">
-        <v>46065.866386678244</v>
+        <v>46065.69972001157</v>
       </c>
       <c r="C27" s="8">
-        <v>46097.553488425925</v>
+        <v>46097.38682175926</v>
       </c>
       <c r="D27" s="8">
-        <v>46097.553490011574</v>
+        <v>46097.3868233449</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>107</v>
@@ -2978,13 +2978,13 @@
         <v>110</v>
       </c>
       <c r="B28" s="5">
-        <v>46065.866386967595</v>
+        <v>46065.69972030092</v>
       </c>
       <c r="C28" s="5">
-        <v>46155.87588472222</v>
+        <v>46155.709218055556</v>
       </c>
       <c r="D28" s="5">
-        <v>46155.87588597222</v>
+        <v>46155.70921930556</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>111</v>
@@ -3039,13 +3039,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46065.866387256945</v>
+        <v>46065.69972059027</v>
       </c>
       <c r="C29" s="8">
-        <v>46122.645094444444</v>
+        <v>46122.47842777778</v>
       </c>
       <c r="D29" s="8">
-        <v>46128.18276325232</v>
+        <v>46128.01609658565</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3104,13 +3104,13 @@
         <v>116</v>
       </c>
       <c r="B30" s="5">
-        <v>46065.86638756945</v>
+        <v>46065.699720902776</v>
       </c>
       <c r="C30" s="5">
-        <v>46097.55455555556</v>
+        <v>46097.38788888889</v>
       </c>
       <c r="D30" s="5">
-        <v>46097.55455702546</v>
+        <v>46097.3878903588</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>117</v>
@@ -3165,13 +3165,13 @@
         <v>119</v>
       </c>
       <c r="B31" s="8">
-        <v>46065.86638787037</v>
+        <v>46065.6997212037</v>
       </c>
       <c r="C31" s="8">
-        <v>46122.64507917824</v>
+        <v>46122.47841251157</v>
       </c>
       <c r="D31" s="8">
-        <v>46122.64508055555</v>
+        <v>46122.47841388889</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>120</v>
@@ -3226,13 +3226,13 @@
         <v>122</v>
       </c>
       <c r="B32" s="5">
-        <v>46065.8663881713</v>
+        <v>46065.69972150463</v>
       </c>
       <c r="C32" s="5">
-        <v>46155.891567349536</v>
+        <v>46155.72490068287</v>
       </c>
       <c r="D32" s="5">
-        <v>46155.89158689815</v>
+        <v>46155.724920231485</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>123</v>
@@ -3291,13 +3291,13 @@
         <v>125</v>
       </c>
       <c r="B33" s="8">
-        <v>46065.86638436343</v>
+        <v>46065.699717696756</v>
       </c>
       <c r="C33" s="8">
-        <v>46139.793677395835</v>
+        <v>46139.627010729164</v>
       </c>
       <c r="D33" s="8">
-        <v>46139.79497809028</v>
+        <v>46139.628311423614</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>126</v>
@@ -3352,13 +3352,13 @@
         <v>128</v>
       </c>
       <c r="B34" s="5">
-        <v>46065.86638475694</v>
+        <v>46065.699718090276</v>
       </c>
       <c r="C34" s="5">
-        <v>46155.89155255787</v>
+        <v>46155.724885891206</v>
       </c>
       <c r="D34" s="5">
-        <v>46155.89155403935</v>
+        <v>46155.724887372686</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>129</v>
@@ -3413,13 +3413,13 @@
         <v>131</v>
       </c>
       <c r="B35" s="8">
-        <v>46065.866385057874</v>
+        <v>46065.6997183912</v>
       </c>
       <c r="C35" s="8">
-        <v>46174.6530503588</v>
+        <v>46174.48638369213</v>
       </c>
       <c r="D35" s="8">
-        <v>46174.65306150463</v>
+        <v>46174.486394837964</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>132</v>
@@ -3478,13 +3478,13 @@
         <v>134</v>
       </c>
       <c r="B36" s="5">
-        <v>46065.866385347224</v>
+        <v>46065.69971868055</v>
       </c>
       <c r="C36" s="5">
-        <v>46097.55406501157</v>
+        <v>46097.38739834491</v>
       </c>
       <c r="D36" s="5">
-        <v>46169.84157347222</v>
+        <v>46169.67490680555</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>135</v>
@@ -3539,13 +3539,13 @@
         <v>137</v>
       </c>
       <c r="B37" s="8">
-        <v>46065.866385636575</v>
+        <v>46065.6997189699</v>
       </c>
       <c r="C37" s="8">
-        <v>46174.652990393515</v>
+        <v>46174.48632372685</v>
       </c>
       <c r="D37" s="8">
-        <v>46174.652992372685</v>
+        <v>46174.48632570602</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>138</v>
@@ -3600,13 +3600,13 @@
         <v>140</v>
       </c>
       <c r="B38" s="5">
-        <v>46065.8663859375</v>
+        <v>46065.69971927084</v>
       </c>
       <c r="C38" s="5">
-        <v>46174.653035868054</v>
+        <v>46174.48636920139</v>
       </c>
       <c r="D38" s="5">
-        <v>46174.653037488424</v>
+        <v>46174.48637082176</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>141</v>
@@ -3661,13 +3661,13 @@
         <v>143</v>
       </c>
       <c r="B39" s="8">
-        <v>46065.866386215275</v>
+        <v>46065.69971954861</v>
       </c>
       <c r="C39" s="8">
-        <v>46118.83673671296</v>
+        <v>46118.6700700463</v>
       </c>
       <c r="D39" s="8">
-        <v>46118.83674979166</v>
+        <v>46118.670083125</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>144</v>
@@ -3726,13 +3726,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46065.86638649306</v>
+        <v>46065.699719826385</v>
       </c>
       <c r="C40" s="5">
-        <v>46118.83650719907</v>
+        <v>46118.669840532406</v>
       </c>
       <c r="D40" s="5">
-        <v>46118.83650899306</v>
+        <v>46118.66984232639</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3787,13 +3787,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46065.86638677084</v>
+        <v>46065.69972010417</v>
       </c>
       <c r="C41" s="8">
-        <v>46118.836723506945</v>
+        <v>46118.670056840274</v>
       </c>
       <c r="D41" s="8">
-        <v>46118.836724988425</v>
+        <v>46118.67005832176</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3848,13 +3848,13 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46065.86638704861</v>
+        <v>46065.69972038195</v>
       </c>
       <c r="C42" s="5">
-        <v>46118.83891240741</v>
+        <v>46118.672245740745</v>
       </c>
       <c r="D42" s="5">
-        <v>46133.19587135417</v>
+        <v>46133.0292046875</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -3913,13 +3913,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46065.86638668981</v>
+        <v>46065.69972002315</v>
       </c>
       <c r="C43" s="8">
-        <v>46118.83884881945</v>
+        <v>46118.672182152775</v>
       </c>
       <c r="D43" s="8">
-        <v>46118.83885034722</v>
+        <v>46118.67218368055</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -3974,13 +3974,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46065.86638707176</v>
+        <v>46065.69972040509</v>
       </c>
       <c r="C44" s="5">
-        <v>46118.838897800924</v>
+        <v>46118.67223113426</v>
       </c>
       <c r="D44" s="5">
-        <v>46118.83889917824</v>
+        <v>46118.67223251157</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4035,11 +4035,11 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46065.866387372684</v>
+        <v>46065.69972070602</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46107.72587710648</v>
+        <v>46107.55921043982</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4084,13 +4084,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46070.744155486114</v>
+        <v>46070.57748881944</v>
       </c>
       <c r="C46" s="5">
-        <v>46107.72579283565</v>
+        <v>46107.559126168984</v>
       </c>
       <c r="D46" s="5">
-        <v>46107.725811412034</v>
+        <v>46107.55914474537</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4149,13 +4149,13 @@
         <v>171</v>
       </c>
       <c r="B47" s="8">
-        <v>46065.86638765046</v>
+        <v>46065.6997209838</v>
       </c>
       <c r="C47" s="8">
-        <v>46107.72585664352</v>
+        <v>46107.55918997685</v>
       </c>
       <c r="D47" s="8">
-        <v>46174.653052037036</v>
+        <v>46174.48638537037</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>166</v>
@@ -4214,13 +4214,13 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46090.74964866898</v>
+        <v>46090.582982002314</v>
       </c>
       <c r="C48" s="5">
-        <v>46107.725927673615</v>
+        <v>46107.55926100694</v>
       </c>
       <c r="D48" s="5">
-        <v>46107.72595083334</v>
+        <v>46107.559284166666</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
@@ -4279,11 +4279,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46090.74982369213</v>
+        <v>46090.58315702547</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46170.18363959491</v>
+        <v>46170.01697292824</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4342,13 +4342,13 @@
         <v>183</v>
       </c>
       <c r="B50" s="5">
-        <v>46065.866387939815</v>
+        <v>46065.69972127315</v>
       </c>
       <c r="C50" s="5">
-        <v>46127.635591377315</v>
+        <v>46127.46892471064</v>
       </c>
       <c r="D50" s="5">
-        <v>46127.63560765046</v>
+        <v>46127.468940983796</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>184</v>
@@ -4395,13 +4395,13 @@
         <v>186</v>
       </c>
       <c r="B51" s="8">
-        <v>46065.86638821759</v>
+        <v>46065.699721550925</v>
       </c>
       <c r="C51" s="8">
-        <v>46122.64297173611</v>
+        <v>46122.476305069446</v>
       </c>
       <c r="D51" s="8">
-        <v>46122.64298887731</v>
+        <v>46122.47632221065</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4460,13 +4460,13 @@
         <v>190</v>
       </c>
       <c r="B52" s="5">
-        <v>46065.86638849537</v>
+        <v>46065.6997218287</v>
       </c>
       <c r="C52" s="5">
-        <v>46127.635570196755</v>
+        <v>46127.4689035301</v>
       </c>
       <c r="D52" s="5">
-        <v>46127.63559171296</v>
+        <v>46127.4689250463</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>191</v>
@@ -4525,13 +4525,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46065.86638876157</v>
+        <v>46065.69972209491</v>
       </c>
       <c r="C53" s="8">
-        <v>46167.59797371528</v>
+        <v>46167.43130704861</v>
       </c>
       <c r="D53" s="8">
-        <v>46167.59798559028</v>
+        <v>46167.43131892361</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4578,13 +4578,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46065.8663890162</v>
+        <v>46065.69972234954</v>
       </c>
       <c r="C54" s="5">
-        <v>46167.545010891205</v>
+        <v>46167.37834422453</v>
       </c>
       <c r="D54" s="5">
-        <v>46167.5450264699</v>
+        <v>46167.378359803246</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4643,13 +4643,13 @@
         <v>202</v>
       </c>
       <c r="B55" s="8">
-        <v>46065.86638931713</v>
+        <v>46065.69972265046</v>
       </c>
       <c r="C55" s="8">
-        <v>46167.59790540509</v>
+        <v>46167.43123873843</v>
       </c>
       <c r="D55" s="8">
-        <v>46167.597926319446</v>
+        <v>46167.431259652774</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>203</v>
@@ -4708,13 +4708,13 @@
         <v>206</v>
       </c>
       <c r="B56" s="5">
-        <v>46065.86638487269</v>
+        <v>46065.699718206015</v>
       </c>
       <c r="C56" s="5">
-        <v>46167.59795763889</v>
+        <v>46167.43129097222</v>
       </c>
       <c r="D56" s="5">
-        <v>46167.59797377315</v>
+        <v>46167.43130710648</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>207</v>
@@ -4773,11 +4773,11 @@
         <v>210</v>
       </c>
       <c r="B57" s="8">
-        <v>46065.86638528935</v>
+        <v>46065.69971862268</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46198.825604212965</v>
+        <v>46198.65893754629</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>184</v>
@@ -4820,13 +4820,13 @@
         <v>212</v>
       </c>
       <c r="B58" s="5">
-        <v>46065.866385601854</v>
+        <v>46065.69971893518</v>
       </c>
       <c r="C58" s="5">
-        <v>46198.824122164355</v>
+        <v>46198.65745549768</v>
       </c>
       <c r="D58" s="5">
-        <v>46198.824139675926</v>
+        <v>46198.657473009254</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>213</v>
@@ -4885,11 +4885,11 @@
         <v>215</v>
       </c>
       <c r="B59" s="8">
-        <v>46065.86638590277</v>
+        <v>46065.699719236116</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46155.89156913194</v>
+        <v>46155.72490246528</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>216</v>
@@ -4948,13 +4948,13 @@
         <v>218</v>
       </c>
       <c r="B60" s="5">
-        <v>46065.86638623843</v>
+        <v>46065.699719571756</v>
       </c>
       <c r="C60" s="5">
-        <v>46198.82559879629</v>
+        <v>46198.658932129634</v>
       </c>
       <c r="D60" s="5">
-        <v>46198.82561377315</v>
+        <v>46198.65894710648</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>219</v>
@@ -5013,11 +5013,11 @@
         <v>221</v>
       </c>
       <c r="B61" s="8">
-        <v>46065.86638653935</v>
+        <v>46065.69971987269</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46130.175001006945</v>
+        <v>46130.00833434028</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>54</v>
@@ -5076,13 +5076,13 @@
         <v>223</v>
       </c>
       <c r="B62" s="5">
-        <v>46065.866386828704</v>
+        <v>46065.69972016204</v>
       </c>
       <c r="C62" s="5">
-        <v>46122.64522528935</v>
+        <v>46122.478558622686</v>
       </c>
       <c r="D62" s="5">
-        <v>46143.17235355324</v>
+        <v>46143.00568688658</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>224</v>
@@ -5141,13 +5141,13 @@
         <v>226</v>
       </c>
       <c r="B63" s="8">
-        <v>46065.8663871412</v>
+        <v>46065.69972047454</v>
       </c>
       <c r="C63" s="8">
-        <v>46197.59918284722</v>
+        <v>46197.43251618056</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.60713444444</v>
+        <v>46197.44046777778</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>227</v>
@@ -5194,13 +5194,13 @@
         <v>229</v>
       </c>
       <c r="B64" s="5">
-        <v>46065.86638744213</v>
+        <v>46065.69972077546</v>
       </c>
       <c r="C64" s="5">
-        <v>46195.866510844906</v>
+        <v>46195.69984417824</v>
       </c>
       <c r="D64" s="5">
-        <v>46195.86652894676</v>
+        <v>46195.69986228009</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>230</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B65" s="8">
-        <v>46065.86638777777</v>
+        <v>46065.699721111116</v>
       </c>
       <c r="C65" s="8">
-        <v>46197.50371587963</v>
+        <v>46197.33704921296</v>
       </c>
       <c r="D65" s="8">
-        <v>46198.82561393519</v>
+        <v>46198.658947268515</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>233</v>
@@ -5324,13 +5324,13 @@
         <v>236</v>
       </c>
       <c r="B66" s="5">
-        <v>46065.86638519676</v>
+        <v>46065.69971853009</v>
       </c>
       <c r="C66" s="5">
-        <v>46197.50377947917</v>
+        <v>46197.3371128125</v>
       </c>
       <c r="D66" s="5">
-        <v>46198.82414078704</v>
+        <v>46198.657474120366</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>237</v>
@@ -5389,11 +5389,11 @@
         <v>240</v>
       </c>
       <c r="B67" s="8">
-        <v>46065.866385601854</v>
+        <v>46065.69971893518</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46197.50378688658</v>
+        <v>46197.337120219905</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>241</v>
@@ -5452,13 +5452,13 @@
         <v>243</v>
       </c>
       <c r="B68" s="5">
-        <v>46065.866385960646</v>
+        <v>46065.69971929398</v>
       </c>
       <c r="C68" s="5">
-        <v>46197.607128483796</v>
+        <v>46197.440461817125</v>
       </c>
       <c r="D68" s="5">
-        <v>46197.60726340278</v>
+        <v>46197.44059673611</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>244</v>
@@ -5517,11 +5517,11 @@
         <v>246</v>
       </c>
       <c r="B69" s="8">
-        <v>46065.86638626158</v>
+        <v>46065.69971959491</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46197.60713396991</v>
+        <v>46197.44046730324</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>
@@ -5578,11 +5578,11 @@
         <v>249</v>
       </c>
       <c r="B70" s="5">
-        <v>46065.8663865625</v>
+        <v>46065.699719895834</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46171.204831423616</v>
+        <v>46171.038164756945</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>182</v>
@@ -5639,11 +5639,11 @@
         <v>251</v>
       </c>
       <c r="B71" s="8">
-        <v>46065.866386863425</v>
+        <v>46065.69972019676</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46090.7553162963</v>
+        <v>46090.58864962963</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>252</v>
@@ -5686,11 +5686,11 @@
         <v>254</v>
       </c>
       <c r="B72" s="5">
-        <v>46065.8663871875</v>
+        <v>46065.69972052083</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46172.17936458334</v>
+        <v>46172.01269791667</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>255</v>
@@ -5747,11 +5747,11 @@
         <v>257</v>
       </c>
       <c r="B73" s="8">
-        <v>46065.86638747685</v>
+        <v>46065.69972081018</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46177.199266296295</v>
+        <v>46177.03259962963</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>258</v>
@@ -5810,11 +5810,11 @@
         <v>261</v>
       </c>
       <c r="B74" s="5">
-        <v>46065.866387766204</v>
+        <v>46065.69972109953</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46178.203143680556</v>
+        <v>46178.036477013884</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>262</v>
@@ -5871,11 +5871,11 @@
         <v>266</v>
       </c>
       <c r="B75" s="8">
-        <v>46065.8663881713</v>
+        <v>46065.69972150463</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46179.18502518519</v>
+        <v>46179.018358518515</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>267</v>
@@ -5932,11 +5932,11 @@
         <v>269</v>
       </c>
       <c r="B76" s="5">
-        <v>46065.866384340276</v>
+        <v>46065.69971767361</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46090.755315567134</v>
+        <v>46090.58864890046</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>270</v>
@@ -5979,11 +5979,11 @@
         <v>272</v>
       </c>
       <c r="B77" s="8">
-        <v>46065.866385138885</v>
+        <v>46065.69971847222</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46190.20534189815</v>
+        <v>46190.03867523148</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>273</v>
@@ -6042,11 +6042,11 @@
         <v>277</v>
       </c>
       <c r="B78" s="5">
-        <v>46065.866385416666</v>
+        <v>46065.699718749995</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46190.205348206015</v>
+        <v>46190.03868153935</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>278</v>
@@ -6105,11 +6105,11 @@
         <v>279</v>
       </c>
       <c r="B79" s="8">
-        <v>46090.75000248842</v>
+        <v>46090.583335821764</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46090.75636387731</v>
+        <v>46090.58969721065</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>280</v>
@@ -6158,11 +6158,11 @@
         <v>282</v>
       </c>
       <c r="B80" s="5">
-        <v>46090.75028462963</v>
+        <v>46090.58361796296</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46190.205342534726</v>
+        <v>46190.038675868054</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>283</v>
@@ -6221,11 +6221,11 @@
         <v>285</v>
       </c>
       <c r="B81" s="8">
-        <v>46090.75057857639</v>
+        <v>46090.58391190972</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46199.19411842593</v>
+        <v>46199.02745175926</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>286</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 13:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -1498,13 +1498,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46065.69972041667</v>
+        <v>46065.86638708333</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55529023148</v>
+        <v>46092.72195689815</v>
       </c>
       <c r="D4" s="5">
-        <v>46133.603651701385</v>
+        <v>46133.77031836806</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1547,13 +1547,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46065.69972087963</v>
+        <v>46065.866387546295</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.555256886575</v>
+        <v>46092.72192355324</v>
       </c>
       <c r="D5" s="8">
-        <v>46092.55529099537</v>
+        <v>46092.72195766204</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1612,13 +1612,13 @@
         <v>33</v>
       </c>
       <c r="B6" s="5">
-        <v>46065.69972138889</v>
+        <v>46065.866388055554</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55525744213</v>
+        <v>46092.721924108795</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55529188657</v>
+        <v>46092.721958553244</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>34</v>
@@ -1677,13 +1677,13 @@
         <v>37</v>
       </c>
       <c r="B7" s="8">
-        <v>46065.69972192129</v>
+        <v>46065.866388587965</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55525792824</v>
+        <v>46092.72192459491</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.555291296296</v>
+        <v>46092.72195796296</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>38</v>
@@ -1742,13 +1742,13 @@
         <v>39</v>
       </c>
       <c r="B8" s="5">
-        <v>46065.69972236111</v>
+        <v>46065.86638902778</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55525841435</v>
+        <v>46092.721925081016</v>
       </c>
       <c r="D8" s="5">
-        <v>46100.6233396412</v>
+        <v>46100.79000630787</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>40</v>
@@ -1807,13 +1807,13 @@
         <v>42</v>
       </c>
       <c r="B9" s="8">
-        <v>46065.69972283565</v>
+        <v>46065.86638950232</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.55525921297</v>
+        <v>46092.721925879625</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.55529192129</v>
+        <v>46092.721958587965</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>43</v>
@@ -1872,11 +1872,11 @@
         <v>44</v>
       </c>
       <c r="B10" s="5">
-        <v>46065.69972333334</v>
+        <v>46065.866389999996</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46097.3876528588</v>
+        <v>46097.55431952546</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -1919,13 +1919,13 @@
         <v>47</v>
       </c>
       <c r="B11" s="8">
-        <v>46065.699723680555</v>
+        <v>46065.86639034722</v>
       </c>
       <c r="C11" s="8">
-        <v>46097.38764217593</v>
+        <v>46097.55430884259</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.38766100694</v>
+        <v>46097.55432767361</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>48</v>
@@ -1984,11 +1984,11 @@
         <v>52</v>
       </c>
       <c r="B12" s="5">
-        <v>46065.69972405092</v>
+        <v>46065.866390717594</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46137.026501875</v>
+        <v>46137.193168541664</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>53</v>
@@ -2047,13 +2047,13 @@
         <v>57</v>
       </c>
       <c r="B13" s="8">
-        <v>46065.69972444444</v>
+        <v>46065.86639111111</v>
       </c>
       <c r="C13" s="8">
-        <v>46114.35589099537</v>
+        <v>46114.522557662036</v>
       </c>
       <c r="D13" s="8">
-        <v>46114.35590498842</v>
+        <v>46114.52257165509</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>58</v>
@@ -2100,13 +2100,13 @@
         <v>60</v>
       </c>
       <c r="B14" s="5">
-        <v>46065.6997184375</v>
+        <v>46065.866385104164</v>
       </c>
       <c r="C14" s="5">
-        <v>46097.38671878472</v>
+        <v>46097.55338545139</v>
       </c>
       <c r="D14" s="5">
-        <v>46097.386736678236</v>
+        <v>46097.55340334491</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>61</v>
@@ -2165,13 +2165,13 @@
         <v>63</v>
       </c>
       <c r="B15" s="8">
-        <v>46065.69972413195</v>
+        <v>46065.86639079861</v>
       </c>
       <c r="C15" s="8">
-        <v>46107.557669560185</v>
+        <v>46107.72433622685</v>
       </c>
       <c r="D15" s="8">
-        <v>46107.55768900463</v>
+        <v>46107.72435567129</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>64</v>
@@ -2230,13 +2230,13 @@
         <v>66</v>
       </c>
       <c r="B16" s="5">
-        <v>46065.6997255787</v>
+        <v>46065.86639224537</v>
       </c>
       <c r="C16" s="5">
-        <v>46107.55771945602</v>
+        <v>46107.72438612269</v>
       </c>
       <c r="D16" s="5">
-        <v>46107.55773701389</v>
+        <v>46107.72440368056</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>67</v>
@@ -2295,13 +2295,13 @@
         <v>69</v>
       </c>
       <c r="B17" s="8">
-        <v>46065.69972638889</v>
+        <v>46065.866393055556</v>
       </c>
       <c r="C17" s="8">
-        <v>46114.35587568287</v>
+        <v>46114.522542349536</v>
       </c>
       <c r="D17" s="8">
-        <v>46114.35589112269</v>
+        <v>46114.52255778935</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>70</v>
@@ -2360,13 +2360,13 @@
         <v>73</v>
       </c>
       <c r="B18" s="5">
-        <v>46065.69972674768</v>
+        <v>46065.866393414355</v>
       </c>
       <c r="C18" s="5">
-        <v>46114.35593553241</v>
+        <v>46114.522602199075</v>
       </c>
       <c r="D18" s="5">
-        <v>46114.355957997686</v>
+        <v>46114.52262466435</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>74</v>
@@ -2413,13 +2413,13 @@
         <v>76</v>
       </c>
       <c r="B19" s="8">
-        <v>46065.69972708334</v>
+        <v>46065.866393749995</v>
       </c>
       <c r="C19" s="8">
-        <v>46097.386754328705</v>
+        <v>46097.55342099537</v>
       </c>
       <c r="D19" s="8">
-        <v>46097.387491747686</v>
+        <v>46097.55415841435</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>77</v>
@@ -2478,13 +2478,13 @@
         <v>79</v>
       </c>
       <c r="B20" s="5">
-        <v>46065.69972747685</v>
+        <v>46065.86639414352</v>
       </c>
       <c r="C20" s="5">
-        <v>46097.38667216436</v>
+        <v>46097.553338831014</v>
       </c>
       <c r="D20" s="5">
-        <v>46107.55769261574</v>
+        <v>46107.72435928241</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>80</v>
@@ -2543,13 +2543,13 @@
         <v>83</v>
       </c>
       <c r="B21" s="8">
-        <v>46065.69972790509</v>
+        <v>46065.866394571756</v>
       </c>
       <c r="C21" s="8">
-        <v>46097.38769659722</v>
+        <v>46097.55436326389</v>
       </c>
       <c r="D21" s="8">
-        <v>46097.38771902778</v>
+        <v>46097.55438569444</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>84</v>
@@ -2608,13 +2608,13 @@
         <v>86</v>
       </c>
       <c r="B22" s="5">
-        <v>46065.69972824074</v>
+        <v>46065.86639490741</v>
       </c>
       <c r="C22" s="5">
-        <v>46113.393608240745</v>
+        <v>46113.5602749074</v>
       </c>
       <c r="D22" s="5">
-        <v>46113.39361032407</v>
+        <v>46113.56027699074</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>87</v>
@@ -2673,13 +2673,13 @@
         <v>90</v>
       </c>
       <c r="B23" s="8">
-        <v>46065.699718703705</v>
+        <v>46065.86638537037</v>
       </c>
       <c r="C23" s="8">
-        <v>46114.35591884259</v>
+        <v>46114.52258550926</v>
       </c>
       <c r="D23" s="8">
-        <v>46114.35640158565</v>
+        <v>46114.52306825231</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>91</v>
@@ -2738,13 +2738,13 @@
         <v>93</v>
       </c>
       <c r="B24" s="5">
-        <v>46065.6997191088</v>
+        <v>46065.86638577546</v>
       </c>
       <c r="C24" s="5">
-        <v>46107.55799318287</v>
+        <v>46107.72465984954</v>
       </c>
       <c r="D24" s="5">
-        <v>46107.55801064815</v>
+        <v>46107.724677314814</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>94</v>
@@ -2803,11 +2803,11 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46065.69971940972</v>
+        <v>46065.86638607639</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="8">
-        <v>46174.486404282405</v>
+        <v>46174.653070949076</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -2852,13 +2852,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46065.69971969907</v>
+        <v>46065.86638636574</v>
       </c>
       <c r="C26" s="5">
-        <v>46155.709235937495</v>
+        <v>46155.875902604166</v>
       </c>
       <c r="D26" s="5">
-        <v>46155.70925018519</v>
+        <v>46155.87591685185</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -2917,13 +2917,13 @@
         <v>106</v>
       </c>
       <c r="B27" s="8">
-        <v>46065.69972001157</v>
+        <v>46065.866386678244</v>
       </c>
       <c r="C27" s="8">
-        <v>46097.38682175926</v>
+        <v>46097.553488425925</v>
       </c>
       <c r="D27" s="8">
-        <v>46097.3868233449</v>
+        <v>46097.553490011574</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>107</v>
@@ -2978,13 +2978,13 @@
         <v>110</v>
       </c>
       <c r="B28" s="5">
-        <v>46065.69972030092</v>
+        <v>46065.866386967595</v>
       </c>
       <c r="C28" s="5">
-        <v>46155.709218055556</v>
+        <v>46155.87588472222</v>
       </c>
       <c r="D28" s="5">
-        <v>46155.70921930556</v>
+        <v>46155.87588597222</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>111</v>
@@ -3039,13 +3039,13 @@
         <v>113</v>
       </c>
       <c r="B29" s="8">
-        <v>46065.69972059027</v>
+        <v>46065.866387256945</v>
       </c>
       <c r="C29" s="8">
-        <v>46122.47842777778</v>
+        <v>46122.645094444444</v>
       </c>
       <c r="D29" s="8">
-        <v>46128.01609658565</v>
+        <v>46128.18276325232</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>114</v>
@@ -3104,13 +3104,13 @@
         <v>116</v>
       </c>
       <c r="B30" s="5">
-        <v>46065.699720902776</v>
+        <v>46065.86638756945</v>
       </c>
       <c r="C30" s="5">
-        <v>46097.38788888889</v>
+        <v>46097.55455555556</v>
       </c>
       <c r="D30" s="5">
-        <v>46097.3878903588</v>
+        <v>46097.55455702546</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>117</v>
@@ -3165,13 +3165,13 @@
         <v>119</v>
       </c>
       <c r="B31" s="8">
-        <v>46065.6997212037</v>
+        <v>46065.86638787037</v>
       </c>
       <c r="C31" s="8">
-        <v>46122.47841251157</v>
+        <v>46122.64507917824</v>
       </c>
       <c r="D31" s="8">
-        <v>46122.47841388889</v>
+        <v>46122.64508055555</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>120</v>
@@ -3226,13 +3226,13 @@
         <v>122</v>
       </c>
       <c r="B32" s="5">
-        <v>46065.69972150463</v>
+        <v>46065.8663881713</v>
       </c>
       <c r="C32" s="5">
-        <v>46155.72490068287</v>
+        <v>46155.891567349536</v>
       </c>
       <c r="D32" s="5">
-        <v>46155.724920231485</v>
+        <v>46155.89158689815</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>123</v>
@@ -3291,13 +3291,13 @@
         <v>125</v>
       </c>
       <c r="B33" s="8">
-        <v>46065.699717696756</v>
+        <v>46065.86638436343</v>
       </c>
       <c r="C33" s="8">
-        <v>46139.627010729164</v>
+        <v>46139.793677395835</v>
       </c>
       <c r="D33" s="8">
-        <v>46139.628311423614</v>
+        <v>46139.79497809028</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>126</v>
@@ -3352,13 +3352,13 @@
         <v>128</v>
       </c>
       <c r="B34" s="5">
-        <v>46065.699718090276</v>
+        <v>46065.86638475694</v>
       </c>
       <c r="C34" s="5">
-        <v>46155.724885891206</v>
+        <v>46155.89155255787</v>
       </c>
       <c r="D34" s="5">
-        <v>46155.724887372686</v>
+        <v>46155.89155403935</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>129</v>
@@ -3413,13 +3413,13 @@
         <v>131</v>
       </c>
       <c r="B35" s="8">
-        <v>46065.6997183912</v>
+        <v>46065.866385057874</v>
       </c>
       <c r="C35" s="8">
-        <v>46174.48638369213</v>
+        <v>46174.6530503588</v>
       </c>
       <c r="D35" s="8">
-        <v>46174.486394837964</v>
+        <v>46174.65306150463</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>132</v>
@@ -3478,13 +3478,13 @@
         <v>134</v>
       </c>
       <c r="B36" s="5">
-        <v>46065.69971868055</v>
+        <v>46065.866385347224</v>
       </c>
       <c r="C36" s="5">
-        <v>46097.38739834491</v>
+        <v>46097.55406501157</v>
       </c>
       <c r="D36" s="5">
-        <v>46169.67490680555</v>
+        <v>46169.84157347222</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>135</v>
@@ -3539,13 +3539,13 @@
         <v>137</v>
       </c>
       <c r="B37" s="8">
-        <v>46065.6997189699</v>
+        <v>46065.866385636575</v>
       </c>
       <c r="C37" s="8">
-        <v>46174.48632372685</v>
+        <v>46174.652990393515</v>
       </c>
       <c r="D37" s="8">
-        <v>46174.48632570602</v>
+        <v>46174.652992372685</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>138</v>
@@ -3600,13 +3600,13 @@
         <v>140</v>
       </c>
       <c r="B38" s="5">
-        <v>46065.69971927084</v>
+        <v>46065.8663859375</v>
       </c>
       <c r="C38" s="5">
-        <v>46174.48636920139</v>
+        <v>46174.653035868054</v>
       </c>
       <c r="D38" s="5">
-        <v>46174.48637082176</v>
+        <v>46174.653037488424</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>141</v>
@@ -3661,13 +3661,13 @@
         <v>143</v>
       </c>
       <c r="B39" s="8">
-        <v>46065.69971954861</v>
+        <v>46065.866386215275</v>
       </c>
       <c r="C39" s="8">
-        <v>46118.6700700463</v>
+        <v>46118.83673671296</v>
       </c>
       <c r="D39" s="8">
-        <v>46118.670083125</v>
+        <v>46118.83674979166</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>144</v>
@@ -3726,13 +3726,13 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46065.699719826385</v>
+        <v>46065.86638649306</v>
       </c>
       <c r="C40" s="5">
-        <v>46118.669840532406</v>
+        <v>46118.83650719907</v>
       </c>
       <c r="D40" s="5">
-        <v>46118.66984232639</v>
+        <v>46118.83650899306</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -3787,13 +3787,13 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46065.69972010417</v>
+        <v>46065.86638677084</v>
       </c>
       <c r="C41" s="8">
-        <v>46118.670056840274</v>
+        <v>46118.836723506945</v>
       </c>
       <c r="D41" s="8">
-        <v>46118.67005832176</v>
+        <v>46118.836724988425</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3848,13 +3848,13 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46065.69972038195</v>
+        <v>46065.86638704861</v>
       </c>
       <c r="C42" s="5">
-        <v>46118.672245740745</v>
+        <v>46118.83891240741</v>
       </c>
       <c r="D42" s="5">
-        <v>46133.0292046875</v>
+        <v>46133.19587135417</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -3913,13 +3913,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46065.69972002315</v>
+        <v>46065.86638668981</v>
       </c>
       <c r="C43" s="8">
-        <v>46118.672182152775</v>
+        <v>46118.83884881945</v>
       </c>
       <c r="D43" s="8">
-        <v>46118.67218368055</v>
+        <v>46118.83885034722</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -3974,13 +3974,13 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46065.69972040509</v>
+        <v>46065.86638707176</v>
       </c>
       <c r="C44" s="5">
-        <v>46118.67223113426</v>
+        <v>46118.838897800924</v>
       </c>
       <c r="D44" s="5">
-        <v>46118.67223251157</v>
+        <v>46118.83889917824</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4035,11 +4035,11 @@
         <v>164</v>
       </c>
       <c r="B45" s="8">
-        <v>46065.69972070602</v>
+        <v>46065.866387372684</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46107.55921043982</v>
+        <v>46107.72587710648</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>165</v>
@@ -4084,13 +4084,13 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46070.57748881944</v>
+        <v>46070.744155486114</v>
       </c>
       <c r="C46" s="5">
-        <v>46107.559126168984</v>
+        <v>46107.72579283565</v>
       </c>
       <c r="D46" s="5">
-        <v>46107.55914474537</v>
+        <v>46107.725811412034</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4149,13 +4149,13 @@
         <v>171</v>
       </c>
       <c r="B47" s="8">
-        <v>46065.6997209838</v>
+        <v>46065.86638765046</v>
       </c>
       <c r="C47" s="8">
-        <v>46107.55918997685</v>
+        <v>46107.72585664352</v>
       </c>
       <c r="D47" s="8">
-        <v>46174.48638537037</v>
+        <v>46174.653052037036</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>166</v>
@@ -4214,13 +4214,13 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46090.582982002314</v>
+        <v>46090.74964866898</v>
       </c>
       <c r="C48" s="5">
-        <v>46107.55926100694</v>
+        <v>46107.725927673615</v>
       </c>
       <c r="D48" s="5">
-        <v>46107.559284166666</v>
+        <v>46107.72595083334</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
@@ -4279,11 +4279,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="8">
-        <v>46090.58315702547</v>
+        <v>46090.74982369213</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46170.01697292824</v>
+        <v>46170.18363959491</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>178</v>
@@ -4342,13 +4342,13 @@
         <v>183</v>
       </c>
       <c r="B50" s="5">
-        <v>46065.69972127315</v>
+        <v>46065.866387939815</v>
       </c>
       <c r="C50" s="5">
-        <v>46127.46892471064</v>
+        <v>46127.635591377315</v>
       </c>
       <c r="D50" s="5">
-        <v>46127.468940983796</v>
+        <v>46127.63560765046</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>184</v>
@@ -4395,13 +4395,13 @@
         <v>186</v>
       </c>
       <c r="B51" s="8">
-        <v>46065.699721550925</v>
+        <v>46065.86638821759</v>
       </c>
       <c r="C51" s="8">
-        <v>46122.476305069446</v>
+        <v>46122.64297173611</v>
       </c>
       <c r="D51" s="8">
-        <v>46122.47632221065</v>
+        <v>46122.64298887731</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>185</v>
@@ -4460,13 +4460,13 @@
         <v>190</v>
       </c>
       <c r="B52" s="5">
-        <v>46065.6997218287</v>
+        <v>46065.86638849537</v>
       </c>
       <c r="C52" s="5">
-        <v>46127.4689035301</v>
+        <v>46127.635570196755</v>
       </c>
       <c r="D52" s="5">
-        <v>46127.4689250463</v>
+        <v>46127.63559171296</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>191</v>
@@ -4525,13 +4525,13 @@
         <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46065.69972209491</v>
+        <v>46065.86638876157</v>
       </c>
       <c r="C53" s="8">
-        <v>46167.43130704861</v>
+        <v>46167.59797371528</v>
       </c>
       <c r="D53" s="8">
-        <v>46167.43131892361</v>
+        <v>46167.59798559028</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>196</v>
@@ -4578,13 +4578,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46065.69972234954</v>
+        <v>46065.8663890162</v>
       </c>
       <c r="C54" s="5">
-        <v>46167.37834422453</v>
+        <v>46167.545010891205</v>
       </c>
       <c r="D54" s="5">
-        <v>46167.378359803246</v>
+        <v>46167.5450264699</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4643,13 +4643,13 @@
         <v>202</v>
       </c>
       <c r="B55" s="8">
-        <v>46065.69972265046</v>
+        <v>46065.86638931713</v>
       </c>
       <c r="C55" s="8">
-        <v>46167.43123873843</v>
+        <v>46167.59790540509</v>
       </c>
       <c r="D55" s="8">
-        <v>46167.431259652774</v>
+        <v>46167.597926319446</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>203</v>
@@ -4708,13 +4708,13 @@
         <v>206</v>
       </c>
       <c r="B56" s="5">
-        <v>46065.699718206015</v>
+        <v>46065.86638487269</v>
       </c>
       <c r="C56" s="5">
-        <v>46167.43129097222</v>
+        <v>46167.59795763889</v>
       </c>
       <c r="D56" s="5">
-        <v>46167.43130710648</v>
+        <v>46167.59797377315</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>207</v>
@@ -4773,11 +4773,11 @@
         <v>210</v>
       </c>
       <c r="B57" s="8">
-        <v>46065.69971862268</v>
+        <v>46065.86638528935</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46198.65893754629</v>
+        <v>46198.825604212965</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>184</v>
@@ -4820,13 +4820,13 @@
         <v>212</v>
       </c>
       <c r="B58" s="5">
-        <v>46065.69971893518</v>
+        <v>46065.866385601854</v>
       </c>
       <c r="C58" s="5">
-        <v>46198.65745549768</v>
+        <v>46198.824122164355</v>
       </c>
       <c r="D58" s="5">
-        <v>46198.657473009254</v>
+        <v>46198.824139675926</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>213</v>
@@ -4885,11 +4885,11 @@
         <v>215</v>
       </c>
       <c r="B59" s="8">
-        <v>46065.699719236116</v>
+        <v>46065.86638590277</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46155.72490246528</v>
+        <v>46155.89156913194</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>216</v>
@@ -4948,13 +4948,13 @@
         <v>218</v>
       </c>
       <c r="B60" s="5">
-        <v>46065.699719571756</v>
+        <v>46065.86638623843</v>
       </c>
       <c r="C60" s="5">
-        <v>46198.658932129634</v>
+        <v>46198.82559879629</v>
       </c>
       <c r="D60" s="5">
-        <v>46198.65894710648</v>
+        <v>46198.82561377315</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>219</v>
@@ -5013,11 +5013,11 @@
         <v>221</v>
       </c>
       <c r="B61" s="8">
-        <v>46065.69971987269</v>
+        <v>46065.86638653935</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46130.00833434028</v>
+        <v>46130.175001006945</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>54</v>
@@ -5076,13 +5076,13 @@
         <v>223</v>
       </c>
       <c r="B62" s="5">
-        <v>46065.69972016204</v>
+        <v>46065.866386828704</v>
       </c>
       <c r="C62" s="5">
-        <v>46122.478558622686</v>
+        <v>46122.64522528935</v>
       </c>
       <c r="D62" s="5">
-        <v>46143.00568688658</v>
+        <v>46143.17235355324</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>224</v>
@@ -5141,13 +5141,13 @@
         <v>226</v>
       </c>
       <c r="B63" s="8">
-        <v>46065.69972047454</v>
+        <v>46065.8663871412</v>
       </c>
       <c r="C63" s="8">
-        <v>46197.43251618056</v>
+        <v>46197.59918284722</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.44046777778</v>
+        <v>46197.60713444444</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>227</v>
@@ -5194,13 +5194,13 @@
         <v>229</v>
       </c>
       <c r="B64" s="5">
-        <v>46065.69972077546</v>
+        <v>46065.86638744213</v>
       </c>
       <c r="C64" s="5">
-        <v>46195.69984417824</v>
+        <v>46195.866510844906</v>
       </c>
       <c r="D64" s="5">
-        <v>46195.69986228009</v>
+        <v>46195.86652894676</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>230</v>
@@ -5259,13 +5259,13 @@
         <v>232</v>
       </c>
       <c r="B65" s="8">
-        <v>46065.699721111116</v>
+        <v>46065.86638777777</v>
       </c>
       <c r="C65" s="8">
-        <v>46197.33704921296</v>
+        <v>46197.50371587963</v>
       </c>
       <c r="D65" s="8">
-        <v>46198.658947268515</v>
+        <v>46198.82561393519</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>233</v>
@@ -5324,13 +5324,13 @@
         <v>236</v>
       </c>
       <c r="B66" s="5">
-        <v>46065.69971853009</v>
+        <v>46065.86638519676</v>
       </c>
       <c r="C66" s="5">
-        <v>46197.3371128125</v>
+        <v>46197.50377947917</v>
       </c>
       <c r="D66" s="5">
-        <v>46198.657474120366</v>
+        <v>46198.82414078704</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>237</v>
@@ -5389,11 +5389,11 @@
         <v>240</v>
       </c>
       <c r="B67" s="8">
-        <v>46065.69971893518</v>
+        <v>46065.866385601854</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46197.337120219905</v>
+        <v>46197.50378688658</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>241</v>
@@ -5452,13 +5452,13 @@
         <v>243</v>
       </c>
       <c r="B68" s="5">
-        <v>46065.69971929398</v>
+        <v>46065.866385960646</v>
       </c>
       <c r="C68" s="5">
-        <v>46197.440461817125</v>
+        <v>46197.607128483796</v>
       </c>
       <c r="D68" s="5">
-        <v>46197.44059673611</v>
+        <v>46197.60726340278</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>244</v>
@@ -5517,11 +5517,11 @@
         <v>246</v>
       </c>
       <c r="B69" s="8">
-        <v>46065.69971959491</v>
+        <v>46065.86638626158</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46197.44046730324</v>
+        <v>46197.60713396991</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>
@@ -5578,11 +5578,11 @@
         <v>249</v>
       </c>
       <c r="B70" s="5">
-        <v>46065.699719895834</v>
+        <v>46065.8663865625</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46171.038164756945</v>
+        <v>46171.204831423616</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>182</v>
@@ -5639,11 +5639,11 @@
         <v>251</v>
       </c>
       <c r="B71" s="8">
-        <v>46065.69972019676</v>
+        <v>46065.866386863425</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46090.58864962963</v>
+        <v>46090.7553162963</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>252</v>
@@ -5686,11 +5686,11 @@
         <v>254</v>
       </c>
       <c r="B72" s="5">
-        <v>46065.69972052083</v>
+        <v>46065.8663871875</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46172.01269791667</v>
+        <v>46172.17936458334</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>255</v>
@@ -5747,11 +5747,11 @@
         <v>257</v>
       </c>
       <c r="B73" s="8">
-        <v>46065.69972081018</v>
+        <v>46065.86638747685</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46177.03259962963</v>
+        <v>46177.199266296295</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>258</v>
@@ -5810,11 +5810,11 @@
         <v>261</v>
       </c>
       <c r="B74" s="5">
-        <v>46065.69972109953</v>
+        <v>46065.866387766204</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46178.036477013884</v>
+        <v>46178.203143680556</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>262</v>
@@ -5871,11 +5871,11 @@
         <v>266</v>
       </c>
       <c r="B75" s="8">
-        <v>46065.69972150463</v>
+        <v>46065.8663881713</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46179.018358518515</v>
+        <v>46179.18502518519</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>267</v>
@@ -5932,11 +5932,11 @@
         <v>269</v>
       </c>
       <c r="B76" s="5">
-        <v>46065.69971767361</v>
+        <v>46065.866384340276</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46090.58864890046</v>
+        <v>46090.755315567134</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>270</v>
@@ -5979,11 +5979,11 @@
         <v>272</v>
       </c>
       <c r="B77" s="8">
-        <v>46065.69971847222</v>
+        <v>46065.866385138885</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46190.03867523148</v>
+        <v>46190.20534189815</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>273</v>
@@ -6042,11 +6042,11 @@
         <v>277</v>
       </c>
       <c r="B78" s="5">
-        <v>46065.699718749995</v>
+        <v>46065.866385416666</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46190.03868153935</v>
+        <v>46190.205348206015</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>278</v>
@@ -6105,11 +6105,11 @@
         <v>279</v>
       </c>
       <c r="B79" s="8">
-        <v>46090.583335821764</v>
+        <v>46090.75000248842</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46090.58969721065</v>
+        <v>46090.75636387731</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>280</v>
@@ -6158,11 +6158,11 @@
         <v>282</v>
       </c>
       <c r="B80" s="5">
-        <v>46090.58361796296</v>
+        <v>46090.75028462963</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46190.038675868054</v>
+        <v>46190.205342534726</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>283</v>
@@ -6221,11 +6221,11 @@
         <v>285</v>
       </c>
       <c r="B81" s="8">
-        <v>46090.58391190972</v>
+        <v>46090.75057857639</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46199.02745175926</v>
+        <v>46199.19411842593</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>286</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 15:00 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46198.825604212965</v>
+        <v>46210.61193216435</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>184</v>
@@ -4893,9 +4893,11 @@
       <c r="B59" s="8">
         <v>46065.86638590277</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46210.61192333333</v>
+      </c>
       <c r="D59" s="8">
-        <v>46155.89156913194</v>
+        <v>46210.611941863426</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>216</v>
@@ -4940,10 +4942,10 @@
         <v>46056</v>
       </c>
       <c r="S59" s="9">
-        <v>0</v>
-      </c>
-      <c r="T59" s="12" t="s">
-        <v>82</v>
+        <v>1</v>
+      </c>
+      <c r="T59" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U59" s="11" t="s">
         <v>32</v>
@@ -5153,7 +5155,7 @@
         <v>46197.59918284722</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.60713444444</v>
+        <v>46210.61246145834</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>227</v>
@@ -5397,9 +5399,11 @@
       <c r="B67" s="8">
         <v>46065.866385601854</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="8">
+        <v>46210.61245306713</v>
+      </c>
       <c r="D67" s="8">
-        <v>46197.50378688658</v>
+        <v>46210.61246942129</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>241</v>
@@ -5444,10 +5448,10 @@
         <v>46154</v>
       </c>
       <c r="S67" s="9">
-        <v>0</v>
-      </c>
-      <c r="T67" s="11" t="s">
-        <v>56</v>
+        <v>1</v>
+      </c>
+      <c r="T67" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U67" s="11" t="s">
         <v>32</v>
@@ -5527,7 +5531,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46197.60713396991</v>
+        <v>46210.61246953704</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>
@@ -5572,8 +5576,8 @@
       <c r="S69" s="9">
         <v>0</v>
       </c>
-      <c r="T69" s="11" t="s">
-        <v>56</v>
+      <c r="T69" s="12" t="s">
+        <v>82</v>
       </c>
       <c r="U69" s="11" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-07 15:32 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -5155,7 +5155,7 @@
         <v>46197.59918284722</v>
       </c>
       <c r="D63" s="8">
-        <v>46210.61246145834</v>
+        <v>46210.640153368055</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>227</v>
@@ -5399,11 +5399,9 @@
       <c r="B67" s="8">
         <v>46065.866385601854</v>
       </c>
-      <c r="C67" s="8">
-        <v>46210.61245306713</v>
-      </c>
+      <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46210.61246942129</v>
+        <v>46210.640305451394</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>241</v>
@@ -5531,7 +5529,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46210.61246953704</v>
+        <v>46210.640152928245</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-09 15:24 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -175,10 +175,10 @@
     <t>Revision tableros pruebas</t>
   </si>
   <si>
-    <t>Recepcion Tableros</t>
-  </si>
-  <si>
-    <t>Ingenieria de servicio:,Embalaje</t>
+    <t xml:space="preserve"> 4197-4198 Recepcion Tableros</t>
+  </si>
+  <si>
+    <t>Ingenieria de servicio:,ot 4196 - 4197-4198 Embalaje</t>
   </si>
   <si>
     <t>Tarea sin iniciar</t>
@@ -376,7 +376,7 @@
     <t>Fabricación Tablero</t>
   </si>
   <si>
-    <t>Tablero,Recepcion Tableros</t>
+    <t>Tablero, 4197-4198 Recepcion Tableros</t>
   </si>
   <si>
     <t>1213249277752978</t>
@@ -541,7 +541,7 @@
     <t>Check Planos</t>
   </si>
   <si>
-    <t>Armado FABRICACIÓN EXTERNA ,Control de calidad Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje sensores y accesorios</t>
+    <t>Armado FABRICACIÓN EXTERNA ,Control de calidad Armado,Montaje motor,Montaje Alabe,ot 4196 Montaje Rodete,Montaje sensores y accesorios</t>
   </si>
   <si>
     <t>1213575386156441</t>
@@ -556,10 +556,10 @@
     <t>francisca.gonzalez@zitron.com</t>
   </si>
   <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
+    <t>ot 4196 Pruebas FAT</t>
+  </si>
+  <si>
+    <t>ot 4196 RE-PINTADO</t>
   </si>
   <si>
     <t>1213249277752993</t>
@@ -646,7 +646,7 @@
     <t>1213249277753000</t>
   </si>
   <si>
-    <t>Recepcion Alabe,Recepcion Rodete,Recepcion Motor,Recepcion Tableros,Recepcion sensores y accesorios</t>
+    <t>Recepcion Alabe,Recepcion Rodete,Recepcion Motor, 4197-4198 Recepcion Tableros,Recepcion sensores y accesorios</t>
   </si>
   <si>
     <t>1213249277753001</t>
@@ -664,7 +664,7 @@
     <t>Recepcion Rodete</t>
   </si>
   <si>
-    <t>Bodega:,Montaje Rodete</t>
+    <t>Bodega:,ot 4196 Montaje Rodete</t>
   </si>
   <si>
     <t>1213249277753003</t>
@@ -697,7 +697,7 @@
     <t>Montaje:</t>
   </si>
   <si>
-    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje sensores y accesorios,Pruebas FAT,RE-PINTADO</t>
+    <t>Revestimiento,Montaje motor,Montaje Alabe,ot 4196 Montaje Rodete,Montaje sensores y accesorios,ot 4196 Pruebas FAT,ot 4196 RE-PINTADO</t>
   </si>
   <si>
     <t>1213249277753007</t>
@@ -706,7 +706,7 @@
     <t>Revestimiento</t>
   </si>
   <si>
-    <t>Montaje Alabe,Montaje Rodete,Montaje:</t>
+    <t>Montaje Alabe,ot 4196 Montaje Rodete,Montaje:</t>
   </si>
   <si>
     <t>1213249277753008</t>
@@ -718,7 +718,7 @@
     <t>Revestimiento,Recepcion Motor,Check Planos</t>
   </si>
   <si>
-    <t>Pruebas FAT,Montaje:</t>
+    <t>ot 4196 Pruebas FAT,Montaje:</t>
   </si>
   <si>
     <t>1213249277753009</t>
@@ -730,13 +730,13 @@
     <t>Recepcion Alabe,Revestimiento,Check Planos</t>
   </si>
   <si>
-    <t>Pruebas FAT,Montaje:,Montaje Rodete</t>
+    <t>ot 4196 Pruebas FAT,Montaje:,ot 4196 Montaje Rodete</t>
   </si>
   <si>
     <t>1213249277753010</t>
   </si>
   <si>
-    <t>Montaje Rodete</t>
+    <t>ot 4196 Montaje Rodete</t>
   </si>
   <si>
     <t>Recepcion Rodete,Revestimiento,Montaje Alabe,Check Planos</t>
@@ -754,7 +754,7 @@
     <t>1213249277753012</t>
   </si>
   <si>
-    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje sensores y accesorios</t>
+    <t>Montaje motor,Montaje Alabe,ot 4196 Montaje Rodete,Montaje sensores y accesorios</t>
   </si>
   <si>
     <t>Montaje:,Check pruebas FAT</t>
@@ -763,7 +763,7 @@
     <t>1213249277753013</t>
   </si>
   <si>
-    <t>Coordinacion Entrega con Cliente,Montaje:</t>
+    <t>ot 4196 - 4197-4198 Coordinacion Entrega con Cliente,Montaje:</t>
   </si>
   <si>
     <t>1213249277753014</t>
@@ -772,13 +772,13 @@
     <t>Logistica:</t>
   </si>
   <si>
-    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
+    <t>ot 4196 - 4197-4198 Coordinacion Entrega con Cliente,ot 4196 - 4197-4198 Embalaje,ot 4196 - 4197-4198 PACKING LIST,ot 4196 - 4197-4198 Despacho</t>
   </si>
   <si>
     <t>1213249277753015</t>
   </si>
   <si>
-    <t>Coordinacion Entrega con Cliente</t>
+    <t>ot 4196 - 4197-4198 Coordinacion Entrega con Cliente</t>
   </si>
   <si>
     <t>Karin Pinto</t>
@@ -787,25 +787,25 @@
     <t>kpinto@zitron.com</t>
   </si>
   <si>
-    <t>Embalaje,Logistica:</t>
+    <t>ot 4196 - 4197-4198 Embalaje,Logistica:</t>
   </si>
   <si>
     <t>1213249277753016</t>
   </si>
   <si>
-    <t>Embalaje</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Revision tableros pruebas</t>
-  </si>
-  <si>
-    <t>PACKING LIST,Logistica:</t>
+    <t>ot 4196 - 4197-4198 Embalaje</t>
+  </si>
+  <si>
+    <t>ot 4196 - 4197-4198 Coordinacion Entrega con Cliente,Revision tableros pruebas</t>
+  </si>
+  <si>
+    <t>ot 4196 - 4197-4198 PACKING LIST,Logistica:</t>
   </si>
   <si>
     <t>1213249277753017</t>
   </si>
   <si>
-    <t>PACKING LIST</t>
+    <t>ot 4196 - 4197-4198 PACKING LIST</t>
   </si>
   <si>
     <t>Nicolás Mol</t>
@@ -814,13 +814,13 @@
     <t>nicolas.mol@zitron.com</t>
   </si>
   <si>
-    <t>Despacho,Logistica:</t>
+    <t>ot 4196 - 4197-4198 Despacho,Logistica:</t>
   </si>
   <si>
     <t>1213249277753018</t>
   </si>
   <si>
-    <t>Despacho</t>
+    <t>ot 4196 - 4197-4198 Despacho</t>
   </si>
   <si>
     <t>Costos,Gestion,Logistica:,Logistica:,instalación Componentes</t>
@@ -847,7 +847,7 @@
     <t>nicolas.tello@zitron.com</t>
   </si>
   <si>
-    <t>Despacho,Analisis de costeo</t>
+    <t>ot 4196 - 4197-4198 Despacho,Analisis de costeo</t>
   </si>
   <si>
     <t>1213249277753022</t>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46137.193168541664</v>
+        <v>46212.62892070602</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>53</v>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46210.61193216435</v>
+        <v>46212.6289187963</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>184</v>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46130.175001006945</v>
+        <v>46212.62895899305</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>54</v>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46211.647106944445</v>
+        <v>46212.628313912035</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>241</v>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46210.640152928245</v>
+        <v>46212.62834962963</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>181</v>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46171.204831423616</v>
+        <v>46212.6283765625</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>182</v>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46210.603462604166</v>
+        <v>46212.62862773148</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>255</v>
@@ -5759,7 +5759,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46177.199266296295</v>
+        <v>46212.62856337963</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>260</v>
@@ -5822,7 +5822,7 @@
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46178.203143680556</v>
+        <v>46212.62864408565</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>264</v>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46179.18502518519</v>
+        <v>46212.62866971065</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>269</v>

</xml_diff>